<commit_message>
Printable Sheets are Ready
</commit_message>
<xml_diff>
--- a/Selenium Cheatsheets/CheatSheet-SeleniumPython.xlsx
+++ b/Selenium Cheatsheets/CheatSheet-SeleniumPython.xlsx
@@ -1,19 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28129"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/939c1bf4b082bbe3/Desktop/Projects/Testing Projects/Python-Pytest-Robot/Automation-Testing-with-Python/Selenium with Python/SeleniumDemo/Selenium Basics/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Lenova\OneDrive\Desktop\TestingDocumentation\Selenium Cheatsheets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="3" documentId="8_{B446F88D-CCF3-4DB6-AA5B-B6A9F6F7BFF2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FD5250AE-6C9C-49CC-83A3-715321387EA0}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{908C06CB-A14D-4A34-92A2-CD0BF61EB3A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{4FB147EA-548A-49CC-AAE9-187A6E48BFCB}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{4FB147EA-548A-49CC-AAE9-187A6E48BFCB}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Selenium" sheetId="1" r:id="rId1"/>
     <sheet name="PyTest" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
@@ -707,7 +707,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4">
+  <fonts count="3">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -727,13 +727,6 @@
       <sz val="10"/>
       <color theme="1"/>
       <name val="Arial Unicode MS"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">

</xml_diff>